<commit_message>
Fix: Sua lai danh sach mua
</commit_message>
<xml_diff>
--- a/hardware/bom/Danh sách mua.xlsx
+++ b/hardware/bom/Danh sách mua.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DOWNLOAD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F255F4B7-4692-4445-8389-BDB8C68A8DA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{046ED9FC-8A3A-40A7-849D-D9219B76ECD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="33">
   <si>
     <t>STT</t>
   </si>
@@ -126,6 +126,15 @@
   </si>
   <si>
     <t>BOM V1</t>
+  </si>
+  <si>
+    <t>BMI</t>
+  </si>
+  <si>
+    <t>SparkFun Photodetector Breakout - MAX30101</t>
+  </si>
+  <si>
+    <t>https://www.sparkfun.com/sparkfun-photodetector-breakout-max30101-qwiic.html?srsltid=AYCX9vLpmM3dGNo5q0W0sWt-nVY---ZxP6iWeWo8p3kjkaVzShJKCGly</t>
   </si>
 </sst>
 </file>
@@ -486,7 +495,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -524,7 +533,7 @@
         <v>1</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>5</v>
+        <v>30</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>24</v>
@@ -542,106 +551,125 @@
         <v>2</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>9</v>
-      </c>
+        <v>31</v>
+      </c>
+      <c r="D5" s="3"/>
       <c r="E5" s="4" t="s">
-        <v>22</v>
+        <v>32</v>
       </c>
       <c r="F5" s="3" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="172.8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" ht="72" x14ac:dyDescent="0.3">
       <c r="A6" s="3">
         <v>3</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F6" s="3" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="39.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" ht="172.8" x14ac:dyDescent="0.3">
       <c r="A7" s="3">
         <v>4</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="F7" s="3" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A8" s="3">
         <v>5</v>
       </c>
       <c r="B8" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A9" s="3">
+        <v>6</v>
+      </c>
+      <c r="B9" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C9" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="D9" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="E8" s="3"/>
-      <c r="F8" s="3" t="s">
+      <c r="E9" s="3"/>
+      <c r="F9" s="3" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A9" s="3">
-        <v>8</v>
-      </c>
-      <c r="B9" s="3" t="s">
+    <row r="10" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A10" s="3">
+        <v>7</v>
+      </c>
+      <c r="B10" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C10" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="D10" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="E9" s="4" t="s">
+      <c r="E10" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="F9" s="3" t="s">
+      <c r="F10" s="3" t="s">
         <v>6</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="E6" r:id="rId1" display="https://shopee.vn/B%E1%BA%A3ng-ph%C3%A1t-tri%E1%BB%83n-ESP32-S3-k%E1%BA%BFt-n%E1%BB%91i-Wi-Fi-v%C3%A0-Bluetooth-ti%E1%BB%87n-l%E1%BB%A3i-ph%C3%B9-h%E1%BB%A3p-cho-nhi%E1%BB%81u-thi%E1%BA%BFt-b%E1%BB%8B-IoT-i.770245757.28004785316?rModelId=236524095032&amp;vItemId=49068017154&amp;vModelId=148037671029&amp;vShopId=1506174776&amp;xptdk=20b54445-c098-4405-90cd-837131d9378d" xr:uid="{4080D198-2166-4DED-9853-A95889AD94F5}"/>
-    <hyperlink ref="E5" r:id="rId2" xr:uid="{8AF3A901-7082-4FEF-98E3-F4636E4AE64E}"/>
-    <hyperlink ref="E4" r:id="rId3" xr:uid="{2DA7207B-CAD9-4FD0-9809-A351A2665643}"/>
-    <hyperlink ref="E9" r:id="rId4" xr:uid="{265C8048-BBD3-473D-9462-F643B7F98F96}"/>
-    <hyperlink ref="E7" r:id="rId5" xr:uid="{72DF11A1-7C76-49DE-88FE-396872F99BD6}"/>
+    <hyperlink ref="E7" r:id="rId1" display="https://shopee.vn/B%E1%BA%A3ng-ph%C3%A1t-tri%E1%BB%83n-ESP32-S3-k%E1%BA%BFt-n%E1%BB%91i-Wi-Fi-v%C3%A0-Bluetooth-ti%E1%BB%87n-l%E1%BB%A3i-ph%C3%B9-h%E1%BB%A3p-cho-nhi%E1%BB%81u-thi%E1%BA%BFt-b%E1%BB%8B-IoT-i.770245757.28004785316?rModelId=236524095032&amp;vItemId=49068017154&amp;vModelId=148037671029&amp;vShopId=1506174776&amp;xptdk=20b54445-c098-4405-90cd-837131d9378d" xr:uid="{4080D198-2166-4DED-9853-A95889AD94F5}"/>
+    <hyperlink ref="E6" r:id="rId2" xr:uid="{8AF3A901-7082-4FEF-98E3-F4636E4AE64E}"/>
+    <hyperlink ref="E10" r:id="rId3" xr:uid="{265C8048-BBD3-473D-9462-F643B7F98F96}"/>
+    <hyperlink ref="E8" r:id="rId4" xr:uid="{72DF11A1-7C76-49DE-88FE-396872F99BD6}"/>
+    <hyperlink ref="E4" r:id="rId5" xr:uid="{2DA7207B-CAD9-4FD0-9809-A351A2665643}"/>
+    <hyperlink ref="E5" r:id="rId6" xr:uid="{D198D75C-B7CC-4F31-A209-AEA9E1C8737A}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>